<commit_message>
Add Phase 3 (Teasing & Affiliate) and Phase 4 (D-Day) to Master Dashboard
Phase 3 (D-7 to D-1): Send PR Box to KOC, TikTok teaser videos,
set up Voucher/Flash Sale, prepare FAQ for customer support.

Phase 4 (D-Day): Simultaneous video push, KOC Affiliate posts,
activate TikTok/Shopee Ads, live chat order processing.

Total tasks: 15 across 4 phases with departments Creative, Booking,
Vận hành, CSKH assigned accordingly.

https://claude.ai/code/session_01HinJjmnohbGJvkYXyXFsu7
</commit_message>
<xml_diff>
--- a/TIAN_Launch_MasterPlan_6Phases.xlsx
+++ b/TIAN_Launch_MasterPlan_6Phases.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -908,6 +908,406 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>GD3-01</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>GĐ3: Teasing &amp; Affiliate</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Gửi PR Box cho KOC (unboxing &amp; review)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Lê Văn C</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>→ Sheet 'GD3_Teasing'</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>GD3-02</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>GĐ3: Teasing &amp; Affiliate</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Creative</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Lên video teaser trên TikTok (countdown, sneak peek)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Trần Thị B</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>→ Sheet 'GD3_Teasing'</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>GD3-03</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>GĐ3: Teasing &amp; Affiliate</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Thiết lập Voucher / Flash Sale trên các sàn</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Hoàng Văn E</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>→ Sheet 'GD3_Teasing'</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>GD3-04</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>GĐ3: Teasing &amp; Affiliate</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>CSKH</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Chuẩn bị FAQ &amp; kịch bản trả lời cho CSKH</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Võ Thị F</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>→ Sheet 'GD3_Teasing'</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>GD4-01</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>GĐ4: D-Day Mở bán bùng nổ</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Creative</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Đồng loạt push video lên TikTok, Reels, YouTube Shorts</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Trần Thị B</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>→ Sheet 'GD4_DDay'</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>GD4-02</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>GĐ4: D-Day Mở bán bùng nổ</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Push KOC lên bài kèm link Affiliate đồng loạt</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Lê Văn C</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>→ Sheet 'GD4_DDay'</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>GD4-03</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>GĐ4: D-Day Mở bán bùng nổ</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Bật TikTok Ads / Shopee Ads chuyển đổi</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn A</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>→ Sheet 'GD4_DDay'</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>GD4-04</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>GĐ4: D-Day Mở bán bùng nổ</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>CSKH</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Trực chat và chốt đơn liên tục (Shopee, Lazada, TikTok)</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Võ Thị F</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>→ Sheet 'GD4_DDay'</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Trạng thái" prompt="Chọn trạng thái" type="list">

</xml_diff>

<commit_message>
Add Phase 5 (Post-launch optimization) and Phase 6 (Evaluation) to Master Dashboard
Phase 5 (D+1 to D+3): ROAS analysis for ads budget, collect 5-star
reviews from early buyers, push seeding posts on Facebook groups.

Phase 6 (D+4 onwards): KOC revenue reconciliation report, calculate
3P KPI bonuses, propose long-term sales strategy.

Master Dashboard now complete with all 6 phases (21 tasks total).

https://claude.ai/code/session_01HinJjmnohbGJvkYXyXFsu7
</commit_message>
<xml_diff>
--- a/TIAN_Launch_MasterPlan_6Phases.xlsx
+++ b/TIAN_Launch_MasterPlan_6Phases.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1308,6 +1308,306 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>GD5-01</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>GĐ5: Tối ưu giữa chiến dịch</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Phân tích số liệu ROAS để điều chỉnh ngân sách Ads</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn A</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>→ Sheet 'GD5_ToiUu'</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>GD5-02</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>GĐ5: Tối ưu giữa chiến dịch</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>CSKH</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Xin đánh giá 5 sao từ khách mua sớm (follow-up)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Võ Thị F</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>→ Sheet 'GD5_ToiUu'</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>GD5-03</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>GĐ5: Tối ưu giữa chiến dịch</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Đẩy thêm bài seeding trên group Facebook</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Trần Thị B</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>→ Sheet 'GD5_ToiUu'</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>GD6-01</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>GĐ6: Đánh giá &amp; Duy trì</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Báo cáo đối soát doanh thu KOC (theo từng KOC)</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Lê Văn C</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>→ Sheet 'GD6_DanhGia'</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>GD6-02</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>GĐ6: Đánh giá &amp; Duy trì</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Tính lương thưởng KPI 3P (Performance, Productivity, Profit)</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Hoàng Văn E</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>→ Sheet 'GD6_DanhGia'</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>GD6-03</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>GĐ6: Đánh giá &amp; Duy trì</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Đề xuất chiến lược duy trì bán hàng dài hạn</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn A</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>→ Sheet 'GD6_DanhGia'</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Trạng thái" prompt="Chọn trạng thái" type="list">

</xml_diff>

<commit_message>
Add Team_Creative and Team_Booking sheets with hyperlinks and KPI columns
- Team_Creative (7 tasks): Content, Creative, Design departments
- Team_Booking (4 tasks): Booking, KOC/PR departments
- Each team sheet has 2 extra columns: [KPI / Yêu cầu đầu ra], [Ghi chú nội bộ]
- Master Dashboard column J has clickable hyperlinks to exact row in team sheet
- Team sheets have back-links to Master Dashboard
- Distinct header colors per team (blue for Creative, orange for Booking)

https://claude.ai/code/session_01HinJjmnohbGJvkYXyXFsu7
</commit_message>
<xml_diff>
--- a/TIAN_Launch_MasterPlan_6Phases.xlsx
+++ b/TIAN_Launch_MasterPlan_6Phases.xlsx
@@ -8,6 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Master Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Team_Creative" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Team_Booking" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0&quot;%&quot;"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +39,14 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -81,6 +89,18 @@
         <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+        <bgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C55A11"/>
+        <bgColor rgb="00C55A11"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -100,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -117,6 +137,9 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -125,6 +148,24 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -652,9 +693,9 @@
       <c r="I3" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD1_Concept'</t>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>→ Team_Creative</t>
         </is>
       </c>
     </row>
@@ -702,207 +743,207 @@
       <c r="I4" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD1_Concept'</t>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>→ Team_Booking</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>GD2-01</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>GĐ2: Sản xuất &amp; Setup</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Chụp ảnh nền trắng / concept cho 2 dòng sản phẩm</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Phạm Thị D</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>2026-04-25</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>To-do</t>
-        </is>
-      </c>
-      <c r="I5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD2_SanXuat'</t>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>→ Team_Creative</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>GD2-02</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>GĐ2: Sản xuất &amp; Setup</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Thiết kế Banner sàn (Shopee, Lazada, TikTok Shop)</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Phạm Thị D</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>2026-04-29</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>To-do</t>
-        </is>
-      </c>
-      <c r="I6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD2_SanXuat'</t>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>→ Team_Creative</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>GD2-03</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>GĐ2: Sản xuất &amp; Setup</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Viết listing chuẩn SEO (tiêu đề, mô tả, bullet points)</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Trần Thị B</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>2026-05-05</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>To-do</t>
-        </is>
-      </c>
-      <c r="I7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD2_SanXuat'</t>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>→ Team_Creative</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>GD2-04</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>GĐ2: Sản xuất &amp; Setup</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>E-commerce</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Đăng sản phẩm lên sàn (Shopee, Lazada, TikTok Shop)</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>Hoàng Văn E</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>2026-05-05</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>To-do</t>
-        </is>
-      </c>
-      <c r="I8" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
         <is>
           <t>→ Sheet 'GD2_SanXuat'</t>
         </is>
@@ -944,7 +985,7 @@
           <t>2026-05-10</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>To-do</t>
         </is>
@@ -952,9 +993,9 @@
       <c r="I9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD3_Teasing'</t>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>→ Team_Booking</t>
         </is>
       </c>
     </row>
@@ -994,7 +1035,7 @@
           <t>2026-05-13</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>To-do</t>
         </is>
@@ -1002,9 +1043,9 @@
       <c r="I10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD3_Teasing'</t>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>→ Team_Creative</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1085,7 @@
           <t>2026-05-13</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="H11" s="8" t="inlineStr">
         <is>
           <t>To-do</t>
         </is>
@@ -1094,7 +1135,7 @@
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>To-do</t>
         </is>
@@ -1109,200 +1150,200 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>GD4-01</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>GĐ4: D-Day Mở bán bùng nổ</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Creative</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>Đồng loạt push video lên TikTok, Reels, YouTube Shorts</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>Trần Thị B</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>To-do</t>
-        </is>
-      </c>
-      <c r="I13" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="10" t="inlineStr">
+        <is>
+          <t>→ Team_Creative</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>GD4-02</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>GĐ4: D-Day Mở bán bùng nổ</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Push KOC lên bài kèm link Affiliate đồng loạt</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Lê Văn C</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="10" t="inlineStr">
+        <is>
+          <t>→ Team_Booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>GD4-03</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>GĐ4: D-Day Mở bán bùng nổ</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Bật TikTok Ads / Shopee Ads chuyển đổi</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn A</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
         <is>
           <t>→ Sheet 'GD4_DDay'</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>GD4-02</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>GD4-04</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>GĐ4: D-Day Mở bán bùng nổ</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Booking</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>Push KOC lên bài kèm link Affiliate đồng loạt</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>Lê Văn C</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>CSKH</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Trực chat và chốt đơn liên tục (Shopee, Lazada, TikTok)</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Võ Thị F</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
-        <is>
-          <t>To-do</t>
-        </is>
-      </c>
-      <c r="I14" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="6" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD4_DDay'</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>GD4-03</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>GĐ4: D-Day Mở bán bùng nổ</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>Vận hành</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Bật TikTok Ads / Shopee Ads chuyển đổi</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>Nguyễn Văn A</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="H15" s="7" t="inlineStr">
-        <is>
-          <t>To-do</t>
-        </is>
-      </c>
-      <c r="I15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="6" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD4_DDay'</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>GD4-04</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>GĐ4: D-Day Mở bán bùng nổ</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>CSKH</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>Trực chat và chốt đơn liên tục (Shopee, Lazada, TikTok)</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>Võ Thị F</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="H16" s="7" t="inlineStr">
-        <is>
-          <t>To-do</t>
-        </is>
-      </c>
-      <c r="I16" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
         <is>
           <t>→ Sheet 'GD4_DDay'</t>
         </is>
@@ -1344,7 +1385,7 @@
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H17" s="8" t="inlineStr">
         <is>
           <t>To-do</t>
         </is>
@@ -1394,7 +1435,7 @@
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H18" s="8" t="inlineStr">
         <is>
           <t>To-do</t>
         </is>
@@ -1444,7 +1485,7 @@
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H19" s="8" t="inlineStr">
         <is>
           <t>To-do</t>
         </is>
@@ -1452,157 +1493,157 @@
       <c r="I19" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD5_ToiUu'</t>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>→ Team_Creative</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>GD6-01</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>GĐ6: Đánh giá &amp; Duy trì</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Booking</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>Báo cáo đối soát doanh thu KOC (theo từng KOC)</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
         <is>
           <t>Lê Văn C</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
-        <is>
-          <t>To-do</t>
-        </is>
-      </c>
-      <c r="I20" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="6" t="inlineStr">
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="10" t="inlineStr">
+        <is>
+          <t>→ Team_Booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>GD6-02</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>GĐ6: Đánh giá &amp; Duy trì</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Tính lương thưởng KPI 3P (Performance, Productivity, Profit)</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Hoàng Văn E</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
         <is>
           <t>→ Sheet 'GD6_DanhGia'</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>GD6-02</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>GD6-03</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>GĐ6: Đánh giá &amp; Duy trì</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>Vận hành</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>Tính lương thưởng KPI 3P (Performance, Productivity, Profit)</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>Hoàng Văn E</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="H21" s="7" t="inlineStr">
-        <is>
-          <t>To-do</t>
-        </is>
-      </c>
-      <c r="I21" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="6" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD6_DanhGia'</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>GD6-03</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>GĐ6: Đánh giá &amp; Duy trì</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>Đề xuất chiến lược duy trì bán hàng dài hạn</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Văn A</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
-        <is>
-          <t>To-do</t>
-        </is>
-      </c>
-      <c r="I22" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" s="6" t="inlineStr">
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="7" t="inlineStr">
         <is>
           <t>→ Sheet 'GD6_DanhGia'</t>
         </is>
@@ -1614,6 +1655,840 @@
       <formula1>"To-do,Doing,Done,Overdue"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="J3" location="Team_Creative!A2" display="→ Team_Creative"/>
+    <hyperlink ref="J4" location="Team_Booking!A2" display="→ Team_Booking"/>
+    <hyperlink ref="J5" location="Team_Creative!A3" display="→ Team_Creative"/>
+    <hyperlink ref="J6" location="Team_Creative!A4" display="→ Team_Creative"/>
+    <hyperlink ref="J7" location="Team_Creative!A5" display="→ Team_Creative"/>
+    <hyperlink ref="J9" location="Team_Booking!A3" display="→ Team_Booking"/>
+    <hyperlink ref="J10" location="Team_Creative!A6" display="→ Team_Creative"/>
+    <hyperlink ref="J13" location="Team_Creative!A7" display="→ Team_Creative"/>
+    <hyperlink ref="J14" location="Team_Booking!A4" display="→ Team_Booking"/>
+    <hyperlink ref="J19" location="Team_Creative!A8" display="→ Team_Creative"/>
+    <hyperlink ref="J20" location="Team_Booking!A5" display="→ Team_Booking"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Mã Task</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Giai đoạn</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Phòng ban</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Hạng mục công việc</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>PIC</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>Ngày bắt đầu</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>Tiến độ (%)</t>
+        </is>
+      </c>
+      <c r="J1" s="11" t="inlineStr">
+        <is>
+          <t>Link Sheet Chi tiết</t>
+        </is>
+      </c>
+      <c r="K1" s="11" t="inlineStr">
+        <is>
+          <t>KPI / Yêu cầu đầu ra</t>
+        </is>
+      </c>
+      <c r="L1" s="11" t="inlineStr">
+        <is>
+          <t>Ghi chú nội bộ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>GD1-02</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>GĐ1: Lên Concept &amp; Chuẩn bị</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>Lên kịch bản outline (video review, seeding post)</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>Trần Thị B</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Doing</t>
+        </is>
+      </c>
+      <c r="I2" s="13" t="n">
+        <v>60</v>
+      </c>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K2" s="12" t="inlineStr">
+        <is>
+          <t>Hoàn thành 3 kịch bản outline được duyệt</t>
+        </is>
+      </c>
+      <c r="L2" s="12" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>GD2-01</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>GĐ2: Sản xuất &amp; Setup</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Chụp ảnh nền trắng / concept cho 2 dòng sản phẩm</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Phạm Thị D</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K3" s="12" t="inlineStr">
+        <is>
+          <t>Bộ 20 ảnh nền trắng + 10 ảnh concept / dòng SP</t>
+        </is>
+      </c>
+      <c r="L3" s="12" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>GD2-02</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>GĐ2: Sản xuất &amp; Setup</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Thiết kế Banner sàn (Shopee, Lazada, TikTok Shop)</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>Phạm Thị D</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K4" s="12" t="inlineStr">
+        <is>
+          <t>6 banner (2 sàn x 3 size) đúng spec, duyệt lần 1</t>
+        </is>
+      </c>
+      <c r="L4" s="12" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>GD2-03</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>GĐ2: Sản xuất &amp; Setup</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Viết listing chuẩn SEO (tiêu đề, mô tả, bullet points)</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Trần Thị B</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K5" s="12" t="inlineStr">
+        <is>
+          <t>Listing đạt điểm SEO ≥ 80 trên tool check</t>
+        </is>
+      </c>
+      <c r="L5" s="12" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>GD3-02</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>GĐ3: Teasing &amp; Affiliate</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Creative</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Lên video teaser trên TikTok (countdown, sneak peek)</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Trần Thị B</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K6" s="12" t="inlineStr">
+        <is>
+          <t>3 video teaser đạt ≥ 50K views trong 48h</t>
+        </is>
+      </c>
+      <c r="L6" s="12" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>GD4-01</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>GĐ4: D-Day Mở bán bùng nổ</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>Creative</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Đồng loạt push video lên TikTok, Reels, YouTube Shorts</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>Trần Thị B</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K7" s="12" t="inlineStr">
+        <is>
+          <t>Tổng views D-Day ≥ 200K, engagement rate ≥ 5%</t>
+        </is>
+      </c>
+      <c r="L7" s="12" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>GD5-03</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>GĐ5: Tối ưu giữa chiến dịch</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Đẩy thêm bài seeding trên group Facebook</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>Trần Thị B</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K8" s="12" t="inlineStr">
+        <is>
+          <t>Đăng ≥ 10 bài seeding, reach ≥ 30K</t>
+        </is>
+      </c>
+      <c r="L8" s="12" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"To-do,Doing,Done,Overdue"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="J2" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="J3" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="J4" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="J5" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="J6" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="J7" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="J8" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Mã Task</t>
+        </is>
+      </c>
+      <c r="B1" s="15" t="inlineStr">
+        <is>
+          <t>Giai đoạn</t>
+        </is>
+      </c>
+      <c r="C1" s="15" t="inlineStr">
+        <is>
+          <t>Phòng ban</t>
+        </is>
+      </c>
+      <c r="D1" s="15" t="inlineStr">
+        <is>
+          <t>Hạng mục công việc</t>
+        </is>
+      </c>
+      <c r="E1" s="15" t="inlineStr">
+        <is>
+          <t>PIC</t>
+        </is>
+      </c>
+      <c r="F1" s="15" t="inlineStr">
+        <is>
+          <t>Ngày bắt đầu</t>
+        </is>
+      </c>
+      <c r="G1" s="15" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="H1" s="15" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="I1" s="15" t="inlineStr">
+        <is>
+          <t>Tiến độ (%)</t>
+        </is>
+      </c>
+      <c r="J1" s="15" t="inlineStr">
+        <is>
+          <t>Link Sheet Chi tiết</t>
+        </is>
+      </c>
+      <c r="K1" s="15" t="inlineStr">
+        <is>
+          <t>KPI / Yêu cầu đầu ra</t>
+        </is>
+      </c>
+      <c r="L1" s="15" t="inlineStr">
+        <is>
+          <t>Ghi chú nội bộ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>GD1-03</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>GĐ1: Lên Concept &amp; Chuẩn bị</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>KOC/PR</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>List danh sách KOC mục tiêu &amp; gửi brief</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>Lê Văn C</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Doing</t>
+        </is>
+      </c>
+      <c r="I2" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K2" s="12" t="inlineStr">
+        <is>
+          <t>List ≥ 15 KOC phù hợp, gửi brief trong 3 ngày</t>
+        </is>
+      </c>
+      <c r="L2" s="12" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>GD3-01</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>GĐ3: Teasing &amp; Affiliate</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Gửi PR Box cho KOC (unboxing &amp; review)</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Lê Văn C</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K3" s="12" t="inlineStr">
+        <is>
+          <t>100% PR Box gửi đúng hạn, có tracking</t>
+        </is>
+      </c>
+      <c r="L3" s="12" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>GD4-02</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>GĐ4: D-Day Mở bán bùng nổ</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Push KOC lên bài kèm link Affiliate đồng loạt</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>Lê Văn C</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K4" s="12" t="inlineStr">
+        <is>
+          <t>≥ 10 KOC đăng bài đúng D-Day, kèm link Affiliate</t>
+        </is>
+      </c>
+      <c r="L4" s="12" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>GD6-01</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>GĐ6: Đánh giá &amp; Duy trì</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Báo cáo đối soát doanh thu KOC (theo từng KOC)</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Lê Văn C</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K5" s="12" t="inlineStr">
+        <is>
+          <t>Báo cáo đối soát hoàn thành trong 3 ngày, sai lệch &lt; 2%</t>
+        </is>
+      </c>
+      <c r="L5" s="12" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"To-do,Doing,Done,Overdue"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="J2" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="J3" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="J4" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="J5" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Team_VanHanh and Team_CSKH sheets with hyperlinks and KPI columns
- Team_VanHanh (5 tasks): Vận hành + E-commerce departments
  KPI: ROAS targets, listing coverage, voucher setup, KPI 3P calc
- Team_CSKH (3 tasks): CSKH department
  KPI: FAQ coverage, response time, 5-star review targets
- All 4 team sheets now have [KPI / Yêu cầu đầu ra] and [Ghi chú nội bộ]
- Master Dashboard hyperlinks updated: 19/21 tasks linked to team sheets
- Each team sheet has distinct header color and back-link to Master Dashboard

https://claude.ai/code/session_01HinJjmnohbGJvkYXyXFsu7
</commit_message>
<xml_diff>
--- a/TIAN_Launch_MasterPlan_6Phases.xlsx
+++ b/TIAN_Launch_MasterPlan_6Phases.xlsx
@@ -10,6 +10,8 @@
     <sheet name="Master Dashboard" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Team_Creative" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Team_Booking" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Team_VanHanh" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Team_CSKH" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -46,7 +48,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -101,6 +103,18 @@
         <bgColor rgb="00C55A11"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00548235"/>
+        <bgColor rgb="00548235"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007030A0"/>
+        <bgColor rgb="007030A0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -120,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -165,6 +179,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -943,9 +963,9 @@
       <c r="I8" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="7" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD2_SanXuat'</t>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>→ Team_VanHanh</t>
         </is>
       </c>
     </row>
@@ -1093,9 +1113,9 @@
       <c r="I11" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD3_Teasing'</t>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>→ Team_VanHanh</t>
         </is>
       </c>
     </row>
@@ -1143,9 +1163,9 @@
       <c r="I12" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD3_Teasing'</t>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>→ Team_CSKH</t>
         </is>
       </c>
     </row>
@@ -1293,9 +1313,9 @@
       <c r="I15" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="J15" s="7" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD4_DDay'</t>
+      <c r="J15" s="10" t="inlineStr">
+        <is>
+          <t>→ Team_VanHanh</t>
         </is>
       </c>
     </row>
@@ -1343,9 +1363,9 @@
       <c r="I16" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="J16" s="7" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD4_DDay'</t>
+      <c r="J16" s="10" t="inlineStr">
+        <is>
+          <t>→ Team_CSKH</t>
         </is>
       </c>
     </row>
@@ -1393,9 +1413,9 @@
       <c r="I17" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD5_ToiUu'</t>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>→ Team_VanHanh</t>
         </is>
       </c>
     </row>
@@ -1443,9 +1463,9 @@
       <c r="I18" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD5_ToiUu'</t>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>→ Team_CSKH</t>
         </is>
       </c>
     </row>
@@ -1593,9 +1613,9 @@
       <c r="I21" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>→ Sheet 'GD6_DanhGia'</t>
+      <c r="J21" s="10" t="inlineStr">
+        <is>
+          <t>→ Team_VanHanh</t>
         </is>
       </c>
     </row>
@@ -1661,12 +1681,20 @@
     <hyperlink ref="J5" location="Team_Creative!A3" display="→ Team_Creative"/>
     <hyperlink ref="J6" location="Team_Creative!A4" display="→ Team_Creative"/>
     <hyperlink ref="J7" location="Team_Creative!A5" display="→ Team_Creative"/>
+    <hyperlink ref="J8" location="Team_VanHanh!A2" display="→ Team_VanHanh"/>
     <hyperlink ref="J9" location="Team_Booking!A3" display="→ Team_Booking"/>
     <hyperlink ref="J10" location="Team_Creative!A6" display="→ Team_Creative"/>
+    <hyperlink ref="J11" location="Team_VanHanh!A3" display="→ Team_VanHanh"/>
+    <hyperlink ref="J12" location="Team_CSKH!A2" display="→ Team_CSKH"/>
     <hyperlink ref="J13" location="Team_Creative!A7" display="→ Team_Creative"/>
     <hyperlink ref="J14" location="Team_Booking!A4" display="→ Team_Booking"/>
+    <hyperlink ref="J15" location="Team_VanHanh!A4" display="→ Team_VanHanh"/>
+    <hyperlink ref="J16" location="Team_CSKH!A3" display="→ Team_CSKH"/>
+    <hyperlink ref="J17" location="Team_VanHanh!A5" display="→ Team_VanHanh"/>
+    <hyperlink ref="J18" location="Team_CSKH!A4" display="→ Team_CSKH"/>
     <hyperlink ref="J19" location="Team_Creative!A8" display="→ Team_Creative"/>
     <hyperlink ref="J20" location="Team_Booking!A5" display="→ Team_Booking"/>
+    <hyperlink ref="J21" location="Team_VanHanh!A6" display="→ Team_VanHanh"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2491,4 +2519,654 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Mã Task</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>Giai đoạn</t>
+        </is>
+      </c>
+      <c r="C1" s="16" t="inlineStr">
+        <is>
+          <t>Phòng ban</t>
+        </is>
+      </c>
+      <c r="D1" s="16" t="inlineStr">
+        <is>
+          <t>Hạng mục công việc</t>
+        </is>
+      </c>
+      <c r="E1" s="16" t="inlineStr">
+        <is>
+          <t>PIC</t>
+        </is>
+      </c>
+      <c r="F1" s="16" t="inlineStr">
+        <is>
+          <t>Ngày bắt đầu</t>
+        </is>
+      </c>
+      <c r="G1" s="16" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="H1" s="16" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="I1" s="16" t="inlineStr">
+        <is>
+          <t>Tiến độ (%)</t>
+        </is>
+      </c>
+      <c r="J1" s="16" t="inlineStr">
+        <is>
+          <t>Link Sheet Chi tiết</t>
+        </is>
+      </c>
+      <c r="K1" s="16" t="inlineStr">
+        <is>
+          <t>KPI / Yêu cầu đầu ra</t>
+        </is>
+      </c>
+      <c r="L1" s="16" t="inlineStr">
+        <is>
+          <t>Ghi chú nội bộ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>GD2-04</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>GĐ2: Sản xuất &amp; Setup</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>Đăng sản phẩm lên sàn (Shopee, Lazada, TikTok Shop)</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>Hoàng Văn E</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I2" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K2" s="12" t="inlineStr">
+        <is>
+          <t>100% sản phẩm lên sàn đúng hạn, listing đầy đủ hình + mô tả</t>
+        </is>
+      </c>
+      <c r="L2" s="12" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>GD3-03</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>GĐ3: Teasing &amp; Affiliate</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Thiết lập Voucher / Flash Sale trên các sàn</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Hoàng Văn E</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K3" s="12" t="inlineStr">
+        <is>
+          <t>Voucher/Flash Sale active trước D-Day 48h, test thành công</t>
+        </is>
+      </c>
+      <c r="L3" s="12" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>GD4-03</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>GĐ4: D-Day Mở bán bùng nổ</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Bật TikTok Ads / Shopee Ads chuyển đổi</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn A</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K4" s="12" t="inlineStr">
+        <is>
+          <t>ROAS Ads D-Day ≥ 3.0, budget burn rate đúng kế hoạch</t>
+        </is>
+      </c>
+      <c r="L4" s="12" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>GD5-01</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>GĐ5: Tối ưu giữa chiến dịch</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Phân tích số liệu ROAS để điều chỉnh ngân sách Ads</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn A</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K5" s="12" t="inlineStr">
+        <is>
+          <t>Báo cáo ROAS trong 24h, đề xuất điều chỉnh ngân sách cụ thể</t>
+        </is>
+      </c>
+      <c r="L5" s="12" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>GD6-02</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>GĐ6: Đánh giá &amp; Duy trì</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Tính lương thưởng KPI 3P (Performance, Productivity, Profit)</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Hoàng Văn E</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K6" s="12" t="inlineStr">
+        <is>
+          <t>Bảng tính KPI 3P hoàn thành, sai số &lt; 1%</t>
+        </is>
+      </c>
+      <c r="L6" s="12" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"To-do,Doing,Done,Overdue"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="J2" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="J3" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="J4" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="J5" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="J6" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Mã Task</t>
+        </is>
+      </c>
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>Giai đoạn</t>
+        </is>
+      </c>
+      <c r="C1" s="17" t="inlineStr">
+        <is>
+          <t>Phòng ban</t>
+        </is>
+      </c>
+      <c r="D1" s="17" t="inlineStr">
+        <is>
+          <t>Hạng mục công việc</t>
+        </is>
+      </c>
+      <c r="E1" s="17" t="inlineStr">
+        <is>
+          <t>PIC</t>
+        </is>
+      </c>
+      <c r="F1" s="17" t="inlineStr">
+        <is>
+          <t>Ngày bắt đầu</t>
+        </is>
+      </c>
+      <c r="G1" s="17" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="H1" s="17" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="I1" s="17" t="inlineStr">
+        <is>
+          <t>Tiến độ (%)</t>
+        </is>
+      </c>
+      <c r="J1" s="17" t="inlineStr">
+        <is>
+          <t>Link Sheet Chi tiết</t>
+        </is>
+      </c>
+      <c r="K1" s="17" t="inlineStr">
+        <is>
+          <t>KPI / Yêu cầu đầu ra</t>
+        </is>
+      </c>
+      <c r="L1" s="17" t="inlineStr">
+        <is>
+          <t>Ghi chú nội bộ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>GD3-04</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>GĐ3: Teasing &amp; Affiliate</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>CSKH</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>Chuẩn bị FAQ &amp; kịch bản trả lời cho CSKH</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>Võ Thị F</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I2" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K2" s="12" t="inlineStr">
+        <is>
+          <t>FAQ ≥ 30 câu, kịch bản chat đạt duyệt trước D-2</t>
+        </is>
+      </c>
+      <c r="L2" s="12" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>GD4-04</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>GĐ4: D-Day Mở bán bùng nổ</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>CSKH</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Trực chat và chốt đơn liên tục (Shopee, Lazada, TikTok)</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Võ Thị F</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K3" s="12" t="inlineStr">
+        <is>
+          <t>Tỷ lệ phản hồi &lt; 5 phút, tỷ lệ chốt đơn ≥ 40%</t>
+        </is>
+      </c>
+      <c r="L3" s="12" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>GD5-02</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>GĐ5: Tối ưu giữa chiến dịch</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>CSKH</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Xin đánh giá 5 sao từ khách mua sớm (follow-up)</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>Võ Thị F</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>To-do</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+      <c r="K4" s="12" t="inlineStr">
+        <is>
+          <t>≥ 50 đánh giá 5 sao trong 3 ngày đầu</t>
+        </is>
+      </c>
+      <c r="L4" s="12" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"To-do,Doing,Done,Overdue"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="J2" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="J3" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="J4" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add KPI_Tracker sheet, Conditional Formatting, and Data Bars - final version
- KPI_Tracker sheet with 5 positions: salary, KPI max, bonus mechanism,
  evaluation %, and auto-calculated bonus formula (=KPI_max * eval%)
- Conditional Formatting on all 5 task sheets:
  - Status column: To-do (grey), Doing (yellow), Done (green), Overdue (red)
  - Progress column: blue Data Bars (0-100%)
- KPI_Tracker: green Data Bar on evaluation column
- Updated To-do status color from blue to grey across all sheets
- Complete file: 6 sheets, 21 tasks, 5 KPI positions, full formatting

https://claude.ai/code/session_01HinJjmnohbGJvkYXyXFsu7
</commit_message>
<xml_diff>
--- a/TIAN_Launch_MasterPlan_6Phases.xlsx
+++ b/TIAN_Launch_MasterPlan_6Phases.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Team_Booking" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Team_VanHanh" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Team_CSKH" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="KPI_Tracker" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -48,7 +49,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -115,6 +116,18 @@
         <bgColor rgb="007030A0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BF8F00"/>
+        <bgColor rgb="00BF8F00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+        <bgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -134,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -157,7 +170,7 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,10 +200,72 @@
     <xf numFmtId="0" fontId="1" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <color rgb="00595959"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D9D9D9"/>
+          <bgColor rgb="00D9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <color rgb="007F6003"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFE699"/>
+          <bgColor rgb="00FFE699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <color rgb="00006100"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+          <bgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -1670,6 +1745,29 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="H2:H100">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"To-do"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Doing"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Done"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"Overdue"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I100">
+    <cfRule type="dataBar" priority="5">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="004472C4"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Trạng thái" prompt="Chọn trạng thái" type="list">
       <formula1>"To-do,Doing,Done,Overdue"</formula1>
@@ -2178,6 +2276,29 @@
       <c r="L8" s="12" t="inlineStr"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="H2:H100">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"To-do"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Doing"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Done"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"Overdue"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I100">
+    <cfRule type="dataBar" priority="5">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="004472C4"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"To-do,Doing,Done,Overdue"</formula1>
@@ -2506,6 +2627,29 @@
       <c r="L5" s="12" t="inlineStr"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="H2:H100">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"To-do"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Doing"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Done"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"Overdue"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I100">
+    <cfRule type="dataBar" priority="5">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="004472C4"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"To-do,Doing,Done,Overdue"</formula1>
@@ -2887,6 +3031,29 @@
       <c r="L6" s="12" t="inlineStr"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="H2:H100">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"To-do"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Doing"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Done"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"Overdue"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I100">
+    <cfRule type="dataBar" priority="5">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="004472C4"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"To-do,Doing,Done,Overdue"</formula1>
@@ -3157,6 +3324,29 @@
       <c r="L4" s="12" t="inlineStr"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="H2:H100">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"To-do"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Doing"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Done"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"Overdue"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I100">
+    <cfRule type="dataBar" priority="5">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="004472C4"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"To-do,Doing,Done,Overdue"</formula1>
@@ -3169,4 +3359,230 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Vị trí</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Lương cứng</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>KPI Trách nhiệm tối đa</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>Cơ chế Thưởng Doanh số</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>Kết quả đánh giá %</t>
+        </is>
+      </c>
+      <c r="F1" s="18" t="inlineStr">
+        <is>
+          <t>Thưởng dự kiến</t>
+        </is>
+      </c>
+      <c r="G1" s="18" t="inlineStr">
+        <is>
+          <t>Điều hướng</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Vận hành sàn (E-commerce)</t>
+        </is>
+      </c>
+      <c r="B2" s="19" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="C2" s="19" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>Từ mốc 1 tỷ: 0.5% DS; 2 tỷ: 0.8% DS; 3 tỷ+: 1% DS</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="n">
+        <v>85</v>
+      </c>
+      <c r="F2" s="19">
+        <f>C2*E2/100</f>
+        <v/>
+      </c>
+      <c r="G2" s="20" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Creative (Content + Design)</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="n">
+        <v>9000000</v>
+      </c>
+      <c r="C3" s="19" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Thưởng cố định theo campaign: 3tr/chiến dịch đạt KPI</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>90</v>
+      </c>
+      <c r="F3" s="19">
+        <f>C3*E3/100</f>
+        <v/>
+      </c>
+      <c r="G3" s="20" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Booking (KOC/PR)</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="C4" s="19" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>2% doanh thu từ link Affiliate KOC quản lý</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>75</v>
+      </c>
+      <c r="F4" s="19">
+        <f>C4*E4/100</f>
+        <v/>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>CSKH (Chăm sóc khách hàng)</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="n">
+        <v>7500000</v>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Thưởng chốt đơn: 5K/đơn chat; 10K/đơn livestream</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>80</v>
+      </c>
+      <c r="F5" s="19">
+        <f>C5*E5/100</f>
+        <v/>
+      </c>
+      <c r="G5" s="20" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Marketing (Chiến lược)</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="C6" s="19" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Thưởng theo ROAS: đạt ≥ 3.0 được 5tr; ≥ 5.0 được 8tr</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>92</v>
+      </c>
+      <c r="F6" s="19">
+        <f>C6*E6/100</f>
+        <v/>
+      </c>
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>← Master Dashboard</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E2:E6">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="0070AD47"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink ref="G2" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="G3" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="G4" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="G5" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+    <hyperlink ref="G6" location="'Master Dashboard'!A1" display="← Master Dashboard"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>